<commit_message>
11 Yıkama formu Excel dosyasında Denim logosu EMS olarak değiştirildi, form kodları EMS
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6foNXTwf1dGzDjULYpfrk
</commit_message>
<xml_diff>
--- a/formlar/4. Yıkama Bölümü (ERTELENDİ)/EMS.WS.RPR.04.05 Boyama Laboratuvarı Daldırma Formu.xlsx
+++ b/formlar/4. Yıkama Bölümü (ERTELENDİ)/EMS.WS.RPR.04.05 Boyama Laboratuvarı Daldırma Formu.xlsx
@@ -172,7 +172,7 @@
     <t>ONAYLAYAN</t>
   </si>
   <si>
-    <t>EG.QA.FRM.04.07</t>
+    <t>EMS.QA.FRM.04.07</t>
   </si>
   <si>
     <t>Style الموديل</t>
@@ -191,7 +191,7 @@
 عينات أختبار الصبغة</t>
   </si>
   <si>
-    <t>EG.WS.RPR.04.05</t>
+    <t>EMS.WS.RPR.04.05</t>
   </si>
   <si>
     <t>Stil Adı:</t>

</xml_diff>